<commit_message>
Updating extensor optimizer with new data
</commit_message>
<xml_diff>
--- a/Testing_Data/2022_02_Festo/Results_table_10mm_pinned_FishScale.xlsx
+++ b/Testing_Data/2022_02_Festo/Results_table_10mm_pinned_FishScale.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben\Documents\GitHub\Bipedal_Robot\Testing_Data\2022_02_Festo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Bipedal_Robot\Testing_Data\2022_02_Festo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCD9C41D-EE08-40E2-ADC0-7BF62F7B7BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B003D7F-4392-4A99-BDDF-B1999C1DD004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{FDAF32CB-2BA8-47E2-927E-3C1E6066A0C3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FDAF32CB-2BA8-47E2-927E-3C1E6066A0C3}"/>
   </bookViews>
   <sheets>
     <sheet name="ExtTest10mm_1" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="53">
   <si>
     <t>Test #</t>
   </si>
@@ -194,6 +194,12 @@
   </si>
   <si>
     <t xml:space="preserve">Origin bracket also </t>
+  </si>
+  <si>
+    <t>min length test</t>
+  </si>
+  <si>
+    <t>max length test</t>
   </si>
 </sst>
 </file>
@@ -774,6 +780,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -781,7 +788,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1213,6 +1219,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1220,7 +1227,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1370,67 +1376,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:trendlineType val="linear"/>
-            <c:dispRSqr val="1"/>
-            <c:dispEq val="1"/>
-            <c:trendlineLbl>
-              <c:layout>
-                <c:manualLayout>
-                  <c:x val="-0.11303399036537215"/>
-                  <c:y val="-1.248096463189626E-2"/>
-                </c:manualLayout>
-              </c:layout>
-              <c:numFmt formatCode="General" sourceLinked="0"/>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="65000"/>
-                          <a:lumOff val="35000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:latin typeface="+mn-lt"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="+mn-cs"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="en-US"/>
-                </a:p>
-              </c:txPr>
-            </c:trendlineLbl>
-          </c:trendline>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-                <a:prstDash val="sysDot"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
             <c:trendlineType val="poly"/>
             <c:order val="3"/>
             <c:dispRSqr val="1"/>
             <c:dispEq val="1"/>
             <c:trendlineLbl>
-              <c:layout>
-                <c:manualLayout>
-                  <c:x val="7.1578872368074545E-2"/>
-                  <c:y val="-0.51961158320556466"/>
-                </c:manualLayout>
-              </c:layout>
               <c:numFmt formatCode="General" sourceLinked="0"/>
               <c:spPr>
                 <a:noFill/>
@@ -1763,6 +1713,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1770,7 +1721,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2285,6 +2235,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2292,7 +2243,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2843,6 +2793,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2850,7 +2801,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3455,6 +3405,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3462,7 +3413,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4132,6 +4082,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -4139,7 +4090,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8154,16 +8104,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>306387</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>415245</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>84137</xdr:rowOff>
+      <xdr:rowOff>40595</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>333904</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>431876</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>112712</xdr:rowOff>
+      <xdr:rowOff>69170</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8660,7 +8610,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DDD6FA0-ED90-4B9F-A1DF-3E2DAEF07409}">
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="3"/>
@@ -9047,9 +8997,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="7:15" x14ac:dyDescent="0.3">
       <c r="G17" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="7:15" x14ac:dyDescent="0.3">
+      <c r="M20" t="s">
+        <v>51</v>
+      </c>
+      <c r="O20" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="7:15" x14ac:dyDescent="0.3">
+      <c r="M21">
+        <f>MIN(C10:X10)</f>
+        <v>385</v>
+      </c>
+      <c r="O21">
+        <f>MAX(C10:X10)</f>
+        <v>430</v>
       </c>
     </row>
   </sheetData>
@@ -9061,7 +9029,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FA6FDC1-BE91-452E-9828-27A0F9CF4E65}">
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="3"/>
@@ -9518,9 +9486,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="7:15" x14ac:dyDescent="0.3">
       <c r="G17" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="7:15" x14ac:dyDescent="0.3">
+      <c r="M20" t="s">
+        <v>51</v>
+      </c>
+      <c r="O20" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="7:15" x14ac:dyDescent="0.3">
+      <c r="M21">
+        <f>MIN(C10:X10)</f>
+        <v>401</v>
+      </c>
+      <c r="O21">
+        <f>MAX(C10:X10)</f>
+        <v>448</v>
       </c>
     </row>
   </sheetData>
@@ -9532,7 +9518,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50982267-BE91-4E95-AD63-2E538907EFD2}">
-  <dimension ref="A1:Y17"/>
+  <dimension ref="A1:Y21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="3"/>
@@ -10215,9 +10201,27 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="7:15" x14ac:dyDescent="0.3">
       <c r="G17" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="7:15" x14ac:dyDescent="0.3">
+      <c r="M20" t="s">
+        <v>51</v>
+      </c>
+      <c r="O20" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="7:15" x14ac:dyDescent="0.3">
+      <c r="M21">
+        <f>MIN(C10:X10)</f>
+        <v>398</v>
+      </c>
+      <c r="O21">
+        <f>MAX(C10:X10)</f>
+        <v>453</v>
       </c>
     </row>
   </sheetData>
@@ -10677,7 +10681,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="8:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
       <c r="H17" t="s">
         <v>21</v>
       </c>
@@ -10685,17 +10689,35 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="8:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B21">
+        <f>MIN(C10:AM10)</f>
+        <v>409</v>
+      </c>
+      <c r="C21">
+        <f>MAX(C10:AM10)</f>
+        <v>460</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
       <c r="L22" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="8:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:14" x14ac:dyDescent="0.3">
       <c r="L23" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="8:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:14" x14ac:dyDescent="0.3">
       <c r="L24" t="s">
         <v>42</v>
       </c>
@@ -10706,7 +10728,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="8:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:14" x14ac:dyDescent="0.3">
       <c r="L25">
         <v>0</v>
       </c>
@@ -10717,7 +10739,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="8:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:14" x14ac:dyDescent="0.3">
       <c r="L26">
         <v>45</v>
       </c>
@@ -10728,12 +10750,12 @@
         <v>48</v>
       </c>
     </row>
-    <row r="30" spans="8:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:14" x14ac:dyDescent="0.3">
       <c r="L30" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="31" spans="8:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:14" x14ac:dyDescent="0.3">
       <c r="L31" t="s">
         <v>49</v>
       </c>
@@ -10752,7 +10774,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6146F73C-E4FC-4324-9793-33EFE048507C}">
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="3"/>
@@ -11347,6 +11369,24 @@
         <v>0</v>
       </c>
     </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B21">
+        <f>MIN(C10:AM10)</f>
+        <v>392.5</v>
+      </c>
+      <c r="C21">
+        <f>MAX(C10:AM10)</f>
+        <v>459</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -11356,7 +11396,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D752D96D-CFF4-4F0D-A512-550321C29C07}">
-  <dimension ref="A1:AJ18"/>
+  <dimension ref="A1:AJ21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="3"/>
@@ -12161,14 +12201,32 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="21:21" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:21" x14ac:dyDescent="0.3">
       <c r="U17" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="21:21" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:21" x14ac:dyDescent="0.3">
       <c r="U18" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="2:21" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="2:21" x14ac:dyDescent="0.3">
+      <c r="B21">
+        <f>MIN(C10:AM10)</f>
+        <v>380</v>
+      </c>
+      <c r="C21">
+        <f>MAX(C10:AM10)</f>
+        <v>438</v>
       </c>
     </row>
   </sheetData>
@@ -12180,7 +12238,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09E5B9E9-F1B4-4DAB-B7CA-9BCB2303132C}">
-  <dimension ref="A1:AJ19"/>
+  <dimension ref="A1:AJ21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="3"/>
@@ -13144,7 +13202,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="10:29" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:29" x14ac:dyDescent="0.3">
       <c r="J17" t="s">
         <v>30</v>
       </c>
@@ -13152,14 +13210,32 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="10:29" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:29" x14ac:dyDescent="0.3">
       <c r="W18" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="10:29" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:29" x14ac:dyDescent="0.3">
       <c r="AC19" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="2:29" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="2:29" x14ac:dyDescent="0.3">
+      <c r="B21">
+        <f>MIN(C10:AM10)</f>
+        <v>398</v>
+      </c>
+      <c r="C21">
+        <f>MAX(C10:AM10)</f>
+        <v>461</v>
       </c>
     </row>
   </sheetData>

</xml_diff>